<commit_message>
Fix clean FORM headcount export and document UI hang
</commit_message>
<xml_diff>
--- a/docs/MP2027/FORM.xlsx
+++ b/docs/MP2027/FORM.xlsx
@@ -17555,9 +17555,7 @@
       <c r="W30" s="189" t="n"/>
     </row>
     <row r="31" ht="13" customFormat="1" customHeight="1" s="207">
-      <c r="B31" s="179" t="n">
-        <v>9114120018</v>
-      </c>
+      <c r="B31" s="179" t="n"/>
       <c r="C31" s="241">
         <f>IFERROR(IF(VLOOKUP($B31,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B31,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -17583,20 +17581,14 @@
         <f>SUM(F31:Q31)</f>
         <v/>
       </c>
-      <c r="S31" s="200" t="inlineStr">
-        <is>
-          <t>この分には間接部門から直接部門に配賦された数字</t>
-        </is>
-      </c>
+      <c r="S31" s="200" t="n"/>
       <c r="T31" s="201" t="n"/>
       <c r="U31" s="189" t="n"/>
       <c r="V31" s="189" t="n"/>
       <c r="W31" s="189" t="n"/>
     </row>
     <row r="32" ht="13" customFormat="1" customHeight="1" s="207">
-      <c r="B32" s="179" t="n">
-        <v>9114120029</v>
-      </c>
+      <c r="B32" s="179" t="n"/>
       <c r="C32" s="241">
         <f>IFERROR(IF(VLOOKUP($B32,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B32,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -17622,20 +17614,14 @@
         <f>SUM(F32:Q32)</f>
         <v/>
       </c>
-      <c r="S32" s="200" t="inlineStr">
-        <is>
-          <t>この分には間接部門から直接部門に配賦された数字</t>
-        </is>
-      </c>
+      <c r="S32" s="200" t="n"/>
       <c r="T32" s="201" t="n"/>
       <c r="U32" s="189" t="n"/>
       <c r="V32" s="189" t="n"/>
       <c r="W32" s="189" t="n"/>
     </row>
     <row r="33" ht="13" customFormat="1" customHeight="1" s="207">
-      <c r="B33" s="179" t="n">
-        <v>9114120030</v>
-      </c>
+      <c r="B33" s="179" t="n"/>
       <c r="C33" s="241">
         <f>IFERROR(IF(VLOOKUP($B33,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B33,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -17661,20 +17647,14 @@
         <f>SUM(F33:Q33)</f>
         <v/>
       </c>
-      <c r="S33" s="200" t="inlineStr">
-        <is>
-          <t>この分には間接部門から直接部門に配賦された数字</t>
-        </is>
-      </c>
+      <c r="S33" s="200" t="n"/>
       <c r="T33" s="201" t="n"/>
       <c r="U33" s="189" t="n"/>
       <c r="V33" s="189" t="n"/>
       <c r="W33" s="189" t="n"/>
     </row>
     <row r="34" ht="13" customFormat="1" customHeight="1" s="207">
-      <c r="B34" s="179" t="n">
-        <v>9114120021</v>
-      </c>
+      <c r="B34" s="179" t="n"/>
       <c r="C34" s="241">
         <f>IFERROR(IF(VLOOKUP($B34,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B34,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -17700,11 +17680,7 @@
         <f>SUM(F34:Q34)</f>
         <v/>
       </c>
-      <c r="S34" s="200" t="inlineStr">
-        <is>
-          <t>この分には間接部門から直接部門に配賦された数字</t>
-        </is>
-      </c>
+      <c r="S34" s="200" t="n"/>
       <c r="T34" s="201" t="n"/>
       <c r="U34" s="189" t="n"/>
       <c r="V34" s="189" t="n"/>
@@ -17745,9 +17721,7 @@
     </row>
     <row r="36" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A36" s="225" t="n"/>
-      <c r="B36" s="179" t="n">
-        <v>5006016260</v>
-      </c>
+      <c r="B36" s="179" t="n"/>
       <c r="C36" s="182">
         <f>IFERROR(IF(VLOOKUP($B36,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B36,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -17773,11 +17747,7 @@
         <f>SUM(F36:Q36)</f>
         <v/>
       </c>
-      <c r="S36" s="200" t="inlineStr">
-        <is>
-          <t>減価償却費（建物）/Khấu hao (Nhà)</t>
-        </is>
-      </c>
+      <c r="S36" s="200" t="n"/>
       <c r="T36" s="201" t="n"/>
       <c r="U36" s="245" t="n"/>
       <c r="V36" s="245" t="n"/>
@@ -17785,9 +17755,7 @@
     </row>
     <row r="37" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A37" s="225" t="n"/>
-      <c r="B37" s="179" t="n">
-        <v>5006016261</v>
-      </c>
+      <c r="B37" s="179" t="n"/>
       <c r="C37" s="182">
         <f>IFERROR(IF(VLOOKUP($B37,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B37,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -17813,11 +17781,7 @@
         <f>SUM(F37:Q37)</f>
         <v/>
       </c>
-      <c r="S37" s="200" t="inlineStr">
-        <is>
-          <t>減価償却費（土地）/Khấu hao (Đất)</t>
-        </is>
-      </c>
+      <c r="S37" s="200" t="n"/>
       <c r="T37" s="201" t="n"/>
       <c r="U37" s="245" t="n"/>
       <c r="V37" s="245" t="n"/>
@@ -17825,9 +17789,7 @@
     </row>
     <row r="38" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A38" s="225" t="n"/>
-      <c r="B38" s="179" t="n">
-        <v>5006016244</v>
-      </c>
+      <c r="B38" s="179" t="n"/>
       <c r="C38" s="182">
         <f>IFERROR(IF(VLOOKUP($B38,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B38,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -17853,11 +17815,7 @@
         <f>SUM(F38:Q38)</f>
         <v/>
       </c>
-      <c r="S38" s="200" t="inlineStr">
-        <is>
-          <t>減価償却費（設備）/Khấu hao (Thiết bị)</t>
-        </is>
-      </c>
+      <c r="S38" s="200" t="n"/>
       <c r="T38" s="201" t="n"/>
       <c r="U38" s="245" t="n"/>
       <c r="V38" s="245" t="n"/>
@@ -17899,9 +17857,7 @@
     </row>
     <row r="40" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A40" s="225" t="n"/>
-      <c r="B40" s="179" t="n">
-        <v>9114120007</v>
-      </c>
+      <c r="B40" s="179" t="n"/>
       <c r="C40" s="182">
         <f>IFERROR(IF(VLOOKUP($B40,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B40,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -17927,11 +17883,7 @@
         <f>SUM(F40:Q40)</f>
         <v/>
       </c>
-      <c r="S40" s="200" t="inlineStr">
-        <is>
-          <t>固定資産金利（建物）/Lãi (Nhà)</t>
-        </is>
-      </c>
+      <c r="S40" s="200" t="n"/>
       <c r="T40" s="201" t="n"/>
       <c r="U40" s="245" t="n"/>
       <c r="V40" s="245" t="n"/>
@@ -17939,9 +17891,7 @@
     </row>
     <row r="41" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A41" s="225" t="n"/>
-      <c r="B41" s="179" t="n">
-        <v>9114120007</v>
-      </c>
+      <c r="B41" s="179" t="n"/>
       <c r="C41" s="182">
         <f>IFERROR(IF(VLOOKUP($B41,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B41,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -17967,11 +17917,7 @@
         <f>SUM(F41:Q41)</f>
         <v/>
       </c>
-      <c r="S41" s="200" t="inlineStr">
-        <is>
-          <t>固定資産金利（土地）/Lãi (Đất)</t>
-        </is>
-      </c>
+      <c r="S41" s="200" t="n"/>
       <c r="T41" s="201" t="n"/>
       <c r="U41" s="245" t="n"/>
       <c r="V41" s="245" t="n"/>
@@ -17979,9 +17925,7 @@
     </row>
     <row r="42" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A42" s="225" t="n"/>
-      <c r="B42" s="179" t="n">
-        <v>9114120007</v>
-      </c>
+      <c r="B42" s="179" t="n"/>
       <c r="C42" s="182">
         <f>IFERROR(IF(VLOOKUP($B42,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B42,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -18007,11 +17951,7 @@
         <f>SUM(F42:Q42)</f>
         <v/>
       </c>
-      <c r="S42" s="200" t="inlineStr">
-        <is>
-          <t>固定資産金利（設備）/Lãi (Thiết bị)</t>
-        </is>
-      </c>
+      <c r="S42" s="200" t="n"/>
       <c r="T42" s="201" t="n"/>
       <c r="U42" s="245" t="n"/>
       <c r="V42" s="245" t="n"/>
@@ -18044,9 +17984,7 @@
     </row>
     <row r="44" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A44" s="225" t="n"/>
-      <c r="B44" s="179" t="n">
-        <v>5005066281</v>
-      </c>
+      <c r="B44" s="179" t="n"/>
       <c r="C44" s="182">
         <f>IFERROR(IF(VLOOKUP($B44,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B44,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -18072,11 +18010,7 @@
         <f>SUM(F44:Q44)</f>
         <v/>
       </c>
-      <c r="S44" s="200" t="inlineStr">
-        <is>
-          <t>電気代/Tiền điện</t>
-        </is>
-      </c>
+      <c r="S44" s="200" t="n"/>
       <c r="T44" s="201" t="n"/>
       <c r="U44" s="245" t="n"/>
       <c r="V44" s="245" t="n"/>
@@ -18084,9 +18018,7 @@
     </row>
     <row r="45" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A45" s="225" t="n"/>
-      <c r="B45" s="179" t="n">
-        <v>5005066282</v>
-      </c>
+      <c r="B45" s="179" t="n"/>
       <c r="C45" s="182">
         <f>IFERROR(IF(VLOOKUP($B45,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B45,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -18112,11 +18044,7 @@
         <f>SUM(F45:Q45)</f>
         <v/>
       </c>
-      <c r="S45" s="200" t="inlineStr">
-        <is>
-          <t>水道代/Tiền nước</t>
-        </is>
-      </c>
+      <c r="S45" s="200" t="n"/>
       <c r="T45" s="201" t="n"/>
       <c r="U45" s="245" t="n"/>
       <c r="V45" s="245" t="n"/>
@@ -18124,9 +18052,7 @@
     </row>
     <row r="46" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A46" s="225" t="n"/>
-      <c r="B46" s="179" t="n">
-        <v>5005056281</v>
-      </c>
+      <c r="B46" s="179" t="n"/>
       <c r="C46" s="182">
         <f>IFERROR(IF(VLOOKUP($B46,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B46,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -18152,11 +18078,7 @@
         <f>SUM(F46:Q46)</f>
         <v/>
       </c>
-      <c r="S46" s="200" t="inlineStr">
-        <is>
-          <t>ガス代/Tiền gas</t>
-        </is>
-      </c>
+      <c r="S46" s="200" t="n"/>
       <c r="T46" s="201" t="n"/>
       <c r="U46" s="245" t="n"/>
       <c r="V46" s="245" t="n"/>
@@ -18198,9 +18120,7 @@
     </row>
     <row r="48" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A48" s="225" t="n"/>
-      <c r="B48" s="179" t="n">
-        <v>5005016372</v>
-      </c>
+      <c r="B48" s="179" t="n"/>
       <c r="C48" s="182">
         <f>IFERROR(IF(VLOOKUP($B48,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B48,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -18226,11 +18146,7 @@
         <f>SUM(F48:Q48)</f>
         <v/>
       </c>
-      <c r="S48" s="200" t="inlineStr">
-        <is>
-          <t>Hand wash</t>
-        </is>
-      </c>
+      <c r="S48" s="200" t="n"/>
       <c r="T48" s="201" t="n"/>
       <c r="U48" s="245" t="n"/>
       <c r="V48" s="245" t="n"/>
@@ -18238,9 +18154,7 @@
     </row>
     <row r="49" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A49" s="225" t="n"/>
-      <c r="B49" s="179" t="n">
-        <v>5005016372</v>
-      </c>
+      <c r="B49" s="179" t="n"/>
       <c r="C49" s="182">
         <f>IFERROR(IF(VLOOKUP($B49,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B49,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -18266,11 +18180,7 @@
         <f>SUM(F49:Q49)</f>
         <v/>
       </c>
-      <c r="S49" s="200" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Toilet paper </t>
-        </is>
-      </c>
+      <c r="S49" s="200" t="n"/>
       <c r="T49" s="201" t="n"/>
       <c r="U49" s="245" t="n"/>
       <c r="V49" s="245" t="n"/>
@@ -18303,9 +18213,7 @@
     </row>
     <row r="51" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A51" s="225" t="n"/>
-      <c r="B51" s="179" t="n">
-        <v>5005246286</v>
-      </c>
+      <c r="B51" s="179" t="n"/>
       <c r="C51" s="182">
         <f>IFERROR(IF(VLOOKUP($B51,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B51,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -18331,11 +18239,7 @@
         <f>SUM(F51:Q51)</f>
         <v/>
       </c>
-      <c r="S51" s="200" t="inlineStr">
-        <is>
-          <t>cleaning fee</t>
-        </is>
-      </c>
+      <c r="S51" s="200" t="n"/>
       <c r="T51" s="201" t="n"/>
       <c r="U51" s="245" t="n"/>
       <c r="V51" s="245" t="n"/>
@@ -18377,9 +18281,7 @@
     </row>
     <row r="53" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A53" s="225" t="n"/>
-      <c r="B53" s="179" t="n">
-        <v>5004086291</v>
-      </c>
+      <c r="B53" s="179" t="n"/>
       <c r="C53" s="182">
         <f>IFERROR(IF(VLOOKUP($B53,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B53,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -18405,11 +18307,7 @@
         <f>SUM(F53:Q53)</f>
         <v/>
       </c>
-      <c r="S53" s="200" t="inlineStr">
-        <is>
-          <t>出向者BUS送迎費/Chi phí xe bus người JP</t>
-        </is>
-      </c>
+      <c r="S53" s="200" t="n"/>
       <c r="T53" s="201" t="n"/>
       <c r="U53" s="245" t="n"/>
       <c r="V53" s="245" t="n"/>
@@ -18417,9 +18315,7 @@
     </row>
     <row r="54" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A54" s="225" t="n"/>
-      <c r="B54" s="179" t="n">
-        <v>5004086291</v>
-      </c>
+      <c r="B54" s="179" t="n"/>
       <c r="C54" s="182">
         <f>IFERROR(IF(VLOOKUP($B54,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B54,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -18445,11 +18341,7 @@
         <f>SUM(F54:Q54)</f>
         <v/>
       </c>
-      <c r="S54" s="200" t="inlineStr">
-        <is>
-          <t>ローカル社BUS送迎費/Chi phí xe bus người VN</t>
-        </is>
-      </c>
+      <c r="S54" s="200" t="n"/>
       <c r="T54" s="201" t="n"/>
       <c r="U54" s="245" t="n"/>
       <c r="V54" s="245" t="n"/>
@@ -18457,9 +18349,7 @@
     </row>
     <row r="55" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A55" s="225" t="n"/>
-      <c r="B55" s="179" t="n">
-        <v>5004086291</v>
-      </c>
+      <c r="B55" s="179" t="n"/>
       <c r="C55" s="182">
         <f>IFERROR(IF(VLOOKUP($B55,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B55,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -18485,11 +18375,7 @@
         <f>SUM(F55:Q55)</f>
         <v/>
       </c>
-      <c r="S55" s="200" t="inlineStr">
-        <is>
-          <t>制服（申請者）/Đồng phục (người yêu cầu)</t>
-        </is>
-      </c>
+      <c r="S55" s="200" t="n"/>
       <c r="T55" s="201" t="n"/>
       <c r="U55" s="245" t="n"/>
       <c r="V55" s="245" t="n"/>
@@ -18497,9 +18383,7 @@
     </row>
     <row r="56" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A56" s="225" t="n"/>
-      <c r="B56" s="179" t="n">
-        <v>5004086291</v>
-      </c>
+      <c r="B56" s="179" t="n"/>
       <c r="C56" s="182">
         <f>IFERROR(IF(VLOOKUP($B56,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B56,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -18525,11 +18409,7 @@
         <f>SUM(F56:Q56)</f>
         <v/>
       </c>
-      <c r="S56" s="200" t="inlineStr">
-        <is>
-          <t>制服(新人）/Đồng phục (người mới)</t>
-        </is>
-      </c>
+      <c r="S56" s="200" t="n"/>
       <c r="T56" s="201" t="n"/>
       <c r="U56" s="245" t="n"/>
       <c r="V56" s="245" t="n"/>
@@ -18537,9 +18417,7 @@
     </row>
     <row r="57" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A57" s="225" t="n"/>
-      <c r="B57" s="179" t="n">
-        <v>5004086291</v>
-      </c>
+      <c r="B57" s="179" t="n"/>
       <c r="C57" s="182">
         <f>IFERROR(IF(VLOOKUP($B57,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B57,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -18565,11 +18443,7 @@
         <f>SUM(F57:Q57)</f>
         <v/>
       </c>
-      <c r="S57" s="200" t="inlineStr">
-        <is>
-          <t>定年の健康診断費/Chi phí khám sức khỏe hàng năm</t>
-        </is>
-      </c>
+      <c r="S57" s="200" t="n"/>
       <c r="T57" s="201" t="n"/>
       <c r="U57" s="245" t="n"/>
       <c r="V57" s="245" t="n"/>
@@ -18577,9 +18451,7 @@
     </row>
     <row r="58" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A58" s="225" t="n"/>
-      <c r="B58" s="179" t="n">
-        <v>5004086291</v>
-      </c>
+      <c r="B58" s="179" t="n"/>
       <c r="C58" s="182">
         <f>IFERROR(IF(VLOOKUP($B58,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B58,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -18605,11 +18477,7 @@
         <f>SUM(F58:Q58)</f>
         <v/>
       </c>
-      <c r="S58" s="200" t="inlineStr">
-        <is>
-          <t>採用の健康診断費/Chi phí khám sức khỏe tuyển dụng</t>
-        </is>
-      </c>
+      <c r="S58" s="200" t="n"/>
       <c r="T58" s="201" t="n"/>
       <c r="U58" s="245" t="n"/>
       <c r="V58" s="245" t="n"/>
@@ -18617,9 +18485,7 @@
     </row>
     <row r="59" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A59" s="225" t="n"/>
-      <c r="B59" s="179" t="n">
-        <v>5004086291</v>
-      </c>
+      <c r="B59" s="179" t="n"/>
       <c r="C59" s="182">
         <f>IFERROR(IF(VLOOKUP($B59,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B59,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -18645,11 +18511,7 @@
         <f>SUM(F59:Q59)</f>
         <v/>
       </c>
-      <c r="S59" s="200" t="inlineStr">
-        <is>
-          <t>誕生日会/Tiền sinh nhật</t>
-        </is>
-      </c>
+      <c r="S59" s="200" t="n"/>
       <c r="T59" s="201" t="n"/>
       <c r="U59" s="245" t="n"/>
       <c r="V59" s="245" t="n"/>
@@ -18657,9 +18519,7 @@
     </row>
     <row r="60" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A60" s="225" t="n"/>
-      <c r="B60" s="179" t="n">
-        <v>5004086291</v>
-      </c>
+      <c r="B60" s="179" t="n"/>
       <c r="C60" s="182">
         <f>IFERROR(IF(VLOOKUP($B60,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B60,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -18685,11 +18545,7 @@
         <f>SUM(F60:Q60)</f>
         <v/>
       </c>
-      <c r="S60" s="200" t="inlineStr">
-        <is>
-          <t>イベント/Sự kiện</t>
-        </is>
-      </c>
+      <c r="S60" s="200" t="n"/>
       <c r="T60" s="201" t="n"/>
       <c r="U60" s="245" t="n"/>
       <c r="V60" s="245" t="n"/>
@@ -18697,9 +18553,7 @@
     </row>
     <row r="61" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A61" s="225" t="n"/>
-      <c r="B61" s="179" t="n">
-        <v>5004086291</v>
-      </c>
+      <c r="B61" s="179" t="n"/>
       <c r="C61" s="182">
         <f>IFERROR(IF(VLOOKUP($B61,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B61,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -18725,11 +18579,7 @@
         <f>SUM(F61:Q61)</f>
         <v/>
       </c>
-      <c r="S61" s="200" t="inlineStr">
-        <is>
-          <t>慶弔金/Tiền hiếu hỷ</t>
-        </is>
-      </c>
+      <c r="S61" s="200" t="n"/>
       <c r="T61" s="201" t="n"/>
       <c r="U61" s="245" t="n"/>
       <c r="V61" s="245" t="n"/>
@@ -18737,9 +18587,7 @@
     </row>
     <row r="62" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A62" s="225" t="n"/>
-      <c r="B62" s="179" t="n">
-        <v>5004086291</v>
-      </c>
+      <c r="B62" s="179" t="n"/>
       <c r="C62" s="182">
         <f>IFERROR(IF(VLOOKUP($B62,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B62,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -18765,11 +18613,7 @@
         <f>SUM(F62:Q62)</f>
         <v/>
       </c>
-      <c r="S62" s="200" t="inlineStr">
-        <is>
-          <t>出向者TAXI送迎/Chi phí taxi người JP</t>
-        </is>
-      </c>
+      <c r="S62" s="200" t="n"/>
       <c r="T62" s="201" t="n"/>
       <c r="U62" s="245" t="n"/>
       <c r="V62" s="245" t="n"/>
@@ -18777,9 +18621,7 @@
     </row>
     <row r="63" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A63" s="225" t="n"/>
-      <c r="B63" s="179" t="n">
-        <v>5004086291</v>
-      </c>
+      <c r="B63" s="179" t="n"/>
       <c r="C63" s="182">
         <f>IFERROR(IF(VLOOKUP($B63,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B63,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -18805,11 +18647,7 @@
         <f>SUM(F63:Q63)</f>
         <v/>
       </c>
-      <c r="S63" s="200" t="inlineStr">
-        <is>
-          <t>ローカル者TAXI送迎費 /Chi phí taxi người VN</t>
-        </is>
-      </c>
+      <c r="S63" s="200" t="n"/>
       <c r="T63" s="201" t="n"/>
       <c r="U63" s="245" t="n"/>
       <c r="V63" s="245" t="n"/>
@@ -18817,9 +18655,7 @@
     </row>
     <row r="64" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A64" s="225" t="n"/>
-      <c r="B64" s="179" t="n">
-        <v>5004086291</v>
-      </c>
+      <c r="B64" s="179" t="n"/>
       <c r="C64" s="182">
         <f>IFERROR(IF(VLOOKUP($B64,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B64,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -18853,9 +18689,7 @@
     </row>
     <row r="65" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A65" s="225" t="n"/>
-      <c r="B65" s="179" t="n">
-        <v>5004086291</v>
-      </c>
+      <c r="B65" s="179" t="n"/>
       <c r="C65" s="182">
         <f>IFERROR(IF(VLOOKUP($B65,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B65,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -18889,9 +18723,7 @@
     </row>
     <row r="66" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A66" s="225" t="n"/>
-      <c r="B66" s="179" t="n">
-        <v>5004086291</v>
-      </c>
+      <c r="B66" s="179" t="n"/>
       <c r="C66" s="182">
         <f>IFERROR(IF(VLOOKUP($B66,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B66,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -18925,9 +18757,7 @@
     </row>
     <row r="67" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A67" s="225" t="n"/>
-      <c r="B67" s="179" t="n">
-        <v>5004086291</v>
-      </c>
+      <c r="B67" s="179" t="n"/>
       <c r="C67" s="182">
         <f>IFERROR(IF(VLOOKUP($B67,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B67,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -18961,9 +18791,7 @@
     </row>
     <row r="68" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A68" s="225" t="n"/>
-      <c r="B68" s="179" t="n">
-        <v>5004086291</v>
-      </c>
+      <c r="B68" s="179" t="n"/>
       <c r="C68" s="182">
         <f>IFERROR(IF(VLOOKUP($B68,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B68,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -18997,9 +18825,7 @@
     </row>
     <row r="69" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A69" s="225" t="n"/>
-      <c r="B69" s="179" t="n">
-        <v>5004086291</v>
-      </c>
+      <c r="B69" s="179" t="n"/>
       <c r="C69" s="182">
         <f>IFERROR(IF(VLOOKUP($B69,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B69,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -19033,9 +18859,7 @@
     </row>
     <row r="70" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A70" s="225" t="n"/>
-      <c r="B70" s="179" t="n">
-        <v>5004086291</v>
-      </c>
+      <c r="B70" s="179" t="n"/>
       <c r="C70" s="182">
         <f>IFERROR(IF(VLOOKUP($B70,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B70,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -19069,9 +18893,7 @@
     </row>
     <row r="71" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A71" s="225" t="n"/>
-      <c r="B71" s="179" t="n">
-        <v>5004086291</v>
-      </c>
+      <c r="B71" s="179" t="n"/>
       <c r="C71" s="182">
         <f>IFERROR(IF(VLOOKUP($B71,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B71,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -19105,9 +18927,7 @@
     </row>
     <row r="72" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A72" s="225" t="n"/>
-      <c r="B72" s="179" t="n">
-        <v>5004086291</v>
-      </c>
+      <c r="B72" s="179" t="n"/>
       <c r="C72" s="182">
         <f>IFERROR(IF(VLOOKUP($B72,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B72,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -19141,9 +18961,7 @@
     </row>
     <row r="73" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A73" s="225" t="n"/>
-      <c r="B73" s="179" t="n">
-        <v>5004086291</v>
-      </c>
+      <c r="B73" s="179" t="n"/>
       <c r="C73" s="182">
         <f>IFERROR(IF(VLOOKUP($B73,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B73,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -19202,9 +19020,7 @@
     </row>
     <row r="75" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A75" s="225" t="n"/>
-      <c r="B75" s="179" t="n">
-        <v>5005246282</v>
-      </c>
+      <c r="B75" s="179" t="n"/>
       <c r="C75" s="182">
         <f>IFERROR(IF(VLOOKUP($B75,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B75,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -19230,11 +19046,7 @@
         <f>SUM(F75:Q75)</f>
         <v/>
       </c>
-      <c r="S75" s="200" t="inlineStr">
-        <is>
-          <t>System Cost (Mail,VPN,R3, Mes,PLM,VPS,…)</t>
-        </is>
-      </c>
+      <c r="S75" s="200" t="n"/>
       <c r="T75" s="201" t="n"/>
       <c r="U75" s="245" t="n"/>
       <c r="V75" s="245" t="n"/>
@@ -19242,9 +19054,7 @@
     </row>
     <row r="76" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A76" s="225" t="n"/>
-      <c r="B76" s="179" t="n">
-        <v>5005246282</v>
-      </c>
+      <c r="B76" s="179" t="n"/>
       <c r="C76" s="182">
         <f>IFERROR(IF(VLOOKUP($B76,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B76,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -19278,9 +19088,7 @@
     </row>
     <row r="77" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A77" s="225" t="n"/>
-      <c r="B77" s="179" t="n">
-        <v>5005246282</v>
-      </c>
+      <c r="B77" s="179" t="n"/>
       <c r="C77" s="182">
         <f>IFERROR(IF(VLOOKUP($B77,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B77,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -19314,9 +19122,7 @@
     </row>
     <row r="78" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A78" s="225" t="n"/>
-      <c r="B78" s="179" t="n">
-        <v>5005246282</v>
-      </c>
+      <c r="B78" s="179" t="n"/>
       <c r="C78" s="182">
         <f>IFERROR(IF(VLOOKUP($B78,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B78,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -19350,9 +19156,7 @@
     </row>
     <row r="79" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A79" s="225" t="n"/>
-      <c r="B79" s="179" t="n">
-        <v>5005246282</v>
-      </c>
+      <c r="B79" s="179" t="n"/>
       <c r="C79" s="182">
         <f>IFERROR(IF(VLOOKUP($B79,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B79,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -19420,9 +19224,7 @@
     </row>
     <row r="81" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A81" s="225" t="n"/>
-      <c r="B81" s="179" t="n">
-        <v>5005246283</v>
-      </c>
+      <c r="B81" s="179" t="n"/>
       <c r="C81" s="182">
         <f>IFERROR(IF(VLOOKUP($B81,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B81,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -19456,9 +19258,7 @@
     </row>
     <row r="82" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A82" s="225" t="n"/>
-      <c r="B82" s="179" t="n">
-        <v>5005246283</v>
-      </c>
+      <c r="B82" s="179" t="n"/>
       <c r="C82" s="182">
         <f>IFERROR(IF(VLOOKUP($B82,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B82,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -19484,11 +19284,7 @@
         <f>SUM(F82:Q82)</f>
         <v/>
       </c>
-      <c r="S82" s="200" t="inlineStr">
-        <is>
-          <t>Officeライセンスのアップグレード費用</t>
-        </is>
-      </c>
+      <c r="S82" s="200" t="n"/>
       <c r="T82" s="201" t="n"/>
       <c r="U82" s="245" t="n"/>
       <c r="V82" s="245" t="n"/>
@@ -19496,9 +19292,7 @@
     </row>
     <row r="83" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A83" s="225" t="n"/>
-      <c r="B83" s="179" t="n">
-        <v>5005246283</v>
-      </c>
+      <c r="B83" s="179" t="n"/>
       <c r="C83" s="182">
         <f>IFERROR(IF(VLOOKUP($B83,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B83,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -19532,9 +19326,7 @@
     </row>
     <row r="84" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A84" s="225" t="n"/>
-      <c r="B84" s="179" t="n">
-        <v>5005246283</v>
-      </c>
+      <c r="B84" s="179" t="n"/>
       <c r="C84" s="182">
         <f>IFERROR(IF(VLOOKUP($B84,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B84,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -19624,9 +19416,7 @@
     </row>
     <row r="87" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A87" s="225" t="n"/>
-      <c r="B87" s="179" t="n">
-        <v>5005246281</v>
-      </c>
+      <c r="B87" s="179" t="n"/>
       <c r="C87" s="182">
         <f>IFERROR(IF(VLOOKUP($B87,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B87,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -19652,11 +19442,7 @@
         <f>SUM(F87:Q87)</f>
         <v/>
       </c>
-      <c r="S87" s="200" t="inlineStr">
-        <is>
-          <t>11月に配賦のPocket Calendar/Lịch bỏ túi phân bổ tháng 11</t>
-        </is>
-      </c>
+      <c r="S87" s="200" t="n"/>
       <c r="T87" s="201" t="n"/>
       <c r="U87" s="245" t="n"/>
       <c r="V87" s="245" t="n"/>
@@ -19664,9 +19450,7 @@
     </row>
     <row r="88" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A88" s="225" t="n"/>
-      <c r="B88" s="179" t="n">
-        <v>5005246281</v>
-      </c>
+      <c r="B88" s="179" t="n"/>
       <c r="C88" s="182">
         <f>IFERROR(IF(VLOOKUP($B88,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B88,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -19692,11 +19476,7 @@
         <f>SUM(F88:Q88)</f>
         <v/>
       </c>
-      <c r="S88" s="200" t="inlineStr">
-        <is>
-          <t>社員証用写真のみ（再発行時）/Chỉ ảnh thẻ nhân viên (trường hợp phát lại)</t>
-        </is>
-      </c>
+      <c r="S88" s="200" t="n"/>
       <c r="T88" s="201" t="n"/>
       <c r="U88" s="245" t="n"/>
       <c r="V88" s="245" t="n"/>
@@ -19729,9 +19509,7 @@
     </row>
     <row r="90" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A90" s="225" t="n"/>
-      <c r="B90" s="179" t="n">
-        <v>5005246281</v>
-      </c>
+      <c r="B90" s="179" t="n"/>
       <c r="C90" s="182">
         <f>IFERROR(IF(VLOOKUP($B90,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B90,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -19757,11 +19535,7 @@
         <f>SUM(F90:Q90)</f>
         <v/>
       </c>
-      <c r="S90" s="200" t="inlineStr">
-        <is>
-          <t>新入社員：名札+写真/Người mới: Thẻ + ảnh</t>
-        </is>
-      </c>
+      <c r="S90" s="200" t="n"/>
       <c r="T90" s="201" t="n"/>
       <c r="U90" s="245" t="n"/>
       <c r="V90" s="245" t="n"/>
@@ -19769,9 +19543,7 @@
     </row>
     <row r="91" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A91" s="225" t="n"/>
-      <c r="B91" s="179" t="n">
-        <v>5005246281</v>
-      </c>
+      <c r="B91" s="179" t="n"/>
       <c r="C91" s="182">
         <f>IFERROR(IF(VLOOKUP($B91,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B91,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -19797,11 +19569,7 @@
         <f>SUM(F91:Q91)</f>
         <v/>
       </c>
-      <c r="S91" s="200" t="inlineStr">
-        <is>
-          <t>新入社員：ﾌｨﾛｿﾌｨ1,2/Người mới: triết lý 1,2</t>
-        </is>
-      </c>
+      <c r="S91" s="200" t="n"/>
       <c r="T91" s="201" t="n"/>
       <c r="U91" s="245" t="n"/>
       <c r="V91" s="245" t="n"/>
@@ -19809,9 +19577,7 @@
     </row>
     <row r="92" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A92" s="225" t="n"/>
-      <c r="B92" s="179" t="n">
-        <v>5005246281</v>
-      </c>
+      <c r="B92" s="179" t="n"/>
       <c r="C92" s="182">
         <f>IFERROR(IF(VLOOKUP($B92,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B92,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -19845,9 +19611,7 @@
     </row>
     <row r="93" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A93" s="225" t="n"/>
-      <c r="B93" s="179" t="n">
-        <v>5005246281</v>
-      </c>
+      <c r="B93" s="179" t="n"/>
       <c r="C93" s="182">
         <f>IFERROR(IF(VLOOKUP($B93,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B93,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -19915,9 +19679,7 @@
     </row>
     <row r="95" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A95" s="225" t="n"/>
-      <c r="B95" s="179" t="n">
-        <v>5005246288</v>
-      </c>
+      <c r="B95" s="179" t="n"/>
       <c r="C95" s="182">
         <f>IFERROR(IF(VLOOKUP($B95,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B95,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -19943,11 +19705,7 @@
         <f>SUM(F95:Q95)</f>
         <v/>
       </c>
-      <c r="S95" s="200" t="inlineStr">
-        <is>
-          <t>新入社員：名札ケース/Người mới: Vỏ thẻ+kẹp</t>
-        </is>
-      </c>
+      <c r="S95" s="200" t="n"/>
       <c r="T95" s="201" t="n"/>
       <c r="U95" s="245" t="n"/>
       <c r="V95" s="245" t="n"/>
@@ -19955,9 +19713,7 @@
     </row>
     <row r="96" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A96" s="225" t="n"/>
-      <c r="B96" s="179" t="n">
-        <v>5005246288</v>
-      </c>
+      <c r="B96" s="179" t="n"/>
       <c r="C96" s="182">
         <f>IFERROR(IF(VLOOKUP($B96,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B96,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -19983,11 +19739,7 @@
         <f>SUM(F96:Q96)</f>
         <v/>
       </c>
-      <c r="S96" s="200" t="inlineStr">
-        <is>
-          <t>新入社員：ペン/Người mới: Bút bi</t>
-        </is>
-      </c>
+      <c r="S96" s="200" t="n"/>
       <c r="T96" s="201" t="n"/>
       <c r="U96" s="245" t="n"/>
       <c r="V96" s="245" t="n"/>
@@ -19995,9 +19747,7 @@
     </row>
     <row r="97" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A97" s="225" t="n"/>
-      <c r="B97" s="179" t="n">
-        <v>5005246288</v>
-      </c>
+      <c r="B97" s="179" t="n"/>
       <c r="C97" s="182">
         <f>IFERROR(IF(VLOOKUP($B97,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B97,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -20023,11 +19773,7 @@
         <f>SUM(F97:Q97)</f>
         <v/>
       </c>
-      <c r="S97" s="200" t="inlineStr">
-        <is>
-          <t>新入社員：ノート（スタッフ用）/Người mới: Sổ tay (Dùng cho nhân viên)</t>
-        </is>
-      </c>
+      <c r="S97" s="200" t="n"/>
       <c r="T97" s="201" t="n"/>
       <c r="U97" s="245" t="n"/>
       <c r="V97" s="245" t="n"/>
@@ -20035,9 +19781,7 @@
     </row>
     <row r="98" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A98" s="225" t="n"/>
-      <c r="B98" s="179" t="n">
-        <v>5005246288</v>
-      </c>
+      <c r="B98" s="179" t="n"/>
       <c r="C98" s="182">
         <f>IFERROR(IF(VLOOKUP($B98,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B98,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -20063,11 +19807,7 @@
         <f>SUM(F98:Q98)</f>
         <v/>
       </c>
-      <c r="S98" s="200" t="inlineStr">
-        <is>
-          <t>新入社員：ノート (G7社員用）/Người mới: Sổ tay (Dùng cho công nhân)</t>
-        </is>
-      </c>
+      <c r="S98" s="200" t="n"/>
       <c r="T98" s="201" t="n"/>
       <c r="U98" s="245" t="n"/>
       <c r="V98" s="245" t="n"/>
@@ -20109,9 +19849,7 @@
     </row>
     <row r="100" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A100" s="225" t="n"/>
-      <c r="B100" s="179" t="n">
-        <v>5005246288</v>
-      </c>
+      <c r="B100" s="179" t="n"/>
       <c r="C100" s="182">
         <f>IFERROR(IF(VLOOKUP($B100,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B100,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -20137,11 +19875,7 @@
         <f>SUM(F100:Q100)</f>
         <v/>
       </c>
-      <c r="S100" s="200" t="inlineStr">
-        <is>
-          <t>Office parts (Ball pen, File, Clamp, Notes, tape etc）</t>
-        </is>
-      </c>
+      <c r="S100" s="200" t="n"/>
       <c r="T100" s="201" t="n"/>
       <c r="U100" s="245" t="n"/>
       <c r="V100" s="245" t="n"/>
@@ -20149,9 +19883,7 @@
     </row>
     <row r="101" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A101" s="225" t="n"/>
-      <c r="B101" s="179" t="n">
-        <v>5005246288</v>
-      </c>
+      <c r="B101" s="179" t="n"/>
       <c r="C101" s="182">
         <f>IFERROR(IF(VLOOKUP($B101,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B101,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -20177,11 +19909,7 @@
         <f>SUM(F101:Q101)</f>
         <v/>
       </c>
-      <c r="S101" s="200" t="inlineStr">
-        <is>
-          <t>Mebius Toner</t>
-        </is>
-      </c>
+      <c r="S101" s="200" t="n"/>
       <c r="T101" s="201" t="n"/>
       <c r="U101" s="245" t="n"/>
       <c r="V101" s="245" t="n"/>
@@ -20189,9 +19917,7 @@
     </row>
     <row r="102" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A102" s="225" t="n"/>
-      <c r="B102" s="179" t="n">
-        <v>5005246288</v>
-      </c>
+      <c r="B102" s="179" t="n"/>
       <c r="C102" s="182">
         <f>IFERROR(IF(VLOOKUP($B102,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B102,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -20217,11 +19943,7 @@
         <f>SUM(F102:Q102)</f>
         <v/>
       </c>
-      <c r="S102" s="200" t="inlineStr">
-        <is>
-          <t>電話機 2台</t>
-        </is>
-      </c>
+      <c r="S102" s="200" t="n"/>
       <c r="T102" s="201" t="n"/>
       <c r="U102" s="245" t="n"/>
       <c r="V102" s="245" t="n"/>
@@ -20229,9 +19951,7 @@
     </row>
     <row r="103" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A103" s="225" t="n"/>
-      <c r="B103" s="179" t="n">
-        <v>5005246288</v>
-      </c>
+      <c r="B103" s="179" t="n"/>
       <c r="C103" s="182">
         <f>IFERROR(IF(VLOOKUP($B103,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B103,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -20299,9 +20019,7 @@
     </row>
     <row r="105" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A105" s="225" t="n"/>
-      <c r="B105" s="179" t="n">
-        <v>5005016372</v>
-      </c>
+      <c r="B105" s="179" t="n"/>
       <c r="C105" s="182">
         <f>IFERROR(IF(VLOOKUP($B105,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B105,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -20327,11 +20045,7 @@
         <f>SUM(F105:Q105)</f>
         <v/>
       </c>
-      <c r="S105" s="200" t="inlineStr">
-        <is>
-          <t>Masks and Glovers</t>
-        </is>
-      </c>
+      <c r="S105" s="200" t="n"/>
       <c r="T105" s="201" t="n"/>
       <c r="U105" s="245" t="n"/>
       <c r="V105" s="245" t="n"/>
@@ -20339,9 +20053,7 @@
     </row>
     <row r="106" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A106" s="225" t="n"/>
-      <c r="B106" s="179" t="n">
-        <v>5005016372</v>
-      </c>
+      <c r="B106" s="179" t="n"/>
       <c r="C106" s="182">
         <f>IFERROR(IF(VLOOKUP($B106,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B106,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -20375,9 +20087,7 @@
     </row>
     <row r="107" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A107" s="225" t="n"/>
-      <c r="B107" s="179" t="n">
-        <v>5005016372</v>
-      </c>
+      <c r="B107" s="179" t="n"/>
       <c r="C107" s="182">
         <f>IFERROR(IF(VLOOKUP($B107,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B107,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -20439,9 +20149,7 @@
     </row>
     <row r="109" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A109" s="225" t="n"/>
-      <c r="B109" s="179" t="n">
-        <v>5005136281</v>
-      </c>
+      <c r="B109" s="179" t="n"/>
       <c r="C109" s="182">
         <f>IFERROR(IF(VLOOKUP($B109,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B109,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -20467,11 +20175,7 @@
         <f>SUM(F109:Q109)</f>
         <v/>
       </c>
-      <c r="S109" s="200" t="inlineStr">
-        <is>
-          <t>Telephone cost</t>
-        </is>
-      </c>
+      <c r="S109" s="200" t="n"/>
       <c r="T109" s="201" t="n"/>
       <c r="U109" s="245" t="n"/>
       <c r="V109" s="245" t="n"/>
@@ -20479,9 +20183,7 @@
     </row>
     <row r="110" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A110" s="225" t="n"/>
-      <c r="B110" s="179" t="n">
-        <v>5005136281</v>
-      </c>
+      <c r="B110" s="179" t="n"/>
       <c r="C110" s="182">
         <f>IFERROR(IF(VLOOKUP($B110,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B110,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -20515,9 +20217,7 @@
     </row>
     <row r="111" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A111" s="225" t="n"/>
-      <c r="B111" s="179" t="n">
-        <v>5005136291</v>
-      </c>
+      <c r="B111" s="179" t="n"/>
       <c r="C111" s="182">
         <f>IFERROR(IF(VLOOKUP($B111,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B111,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -20543,11 +20243,7 @@
         <f>SUM(F111:Q111)</f>
         <v/>
       </c>
-      <c r="S111" s="200" t="inlineStr">
-        <is>
-          <t>書類郵送費/Chi phí gửi giấy tờ</t>
-        </is>
-      </c>
+      <c r="S111" s="200" t="n"/>
       <c r="T111" s="201" t="n"/>
       <c r="U111" s="245" t="n"/>
       <c r="V111" s="245" t="n"/>
@@ -20617,9 +20313,7 @@
     </row>
     <row r="114" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A114" s="225" t="n"/>
-      <c r="B114" s="179" t="n">
-        <v>5005026371</v>
-      </c>
+      <c r="B114" s="179" t="n"/>
       <c r="C114" s="182">
         <f>IFERROR(IF(VLOOKUP($B114,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B114,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -20645,11 +20339,7 @@
         <f>SUM(F114:Q114)</f>
         <v/>
       </c>
-      <c r="S114" s="200" t="inlineStr">
-        <is>
-          <t>RAM購入</t>
-        </is>
-      </c>
+      <c r="S114" s="200" t="n"/>
       <c r="T114" s="201" t="n"/>
       <c r="U114" s="245" t="n"/>
       <c r="V114" s="245" t="n"/>
@@ -20657,9 +20347,7 @@
     </row>
     <row r="115" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A115" s="225" t="n"/>
-      <c r="B115" s="179" t="n">
-        <v>5005026371</v>
-      </c>
+      <c r="B115" s="179" t="n"/>
       <c r="C115" s="182">
         <f>IFERROR(IF(VLOOKUP($B115,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B115,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -20685,11 +20373,7 @@
         <f>SUM(F115:Q115)</f>
         <v/>
       </c>
-      <c r="S115" s="200" t="inlineStr">
-        <is>
-          <t>4月棚購入/Tonner 箱購入</t>
-        </is>
-      </c>
+      <c r="S115" s="200" t="n"/>
       <c r="T115" s="201" t="n"/>
       <c r="U115" s="245" t="n"/>
       <c r="V115" s="245" t="n"/>
@@ -20697,9 +20381,7 @@
     </row>
     <row r="116" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A116" s="225" t="n"/>
-      <c r="B116" s="179" t="n">
-        <v>5005026371</v>
-      </c>
+      <c r="B116" s="179" t="n"/>
       <c r="C116" s="182">
         <f>IFERROR(IF(VLOOKUP($B116,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B116,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -20725,11 +20407,7 @@
         <f>SUM(F116:Q116)</f>
         <v/>
       </c>
-      <c r="S116" s="200" t="inlineStr">
-        <is>
-          <t>Virgo 機 3台(2台残り）</t>
-        </is>
-      </c>
+      <c r="S116" s="200" t="n"/>
       <c r="T116" s="201" t="n"/>
       <c r="U116" s="245" t="n"/>
       <c r="V116" s="245" t="n"/>
@@ -20737,9 +20415,7 @@
     </row>
     <row r="117" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A117" s="225" t="n"/>
-      <c r="B117" s="179" t="n">
-        <v>5005026371</v>
-      </c>
+      <c r="B117" s="179" t="n"/>
       <c r="C117" s="182">
         <f>IFERROR(IF(VLOOKUP($B117,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B117,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -20765,11 +20441,7 @@
         <f>SUM(F117:Q117)</f>
         <v/>
       </c>
-      <c r="S117" s="200" t="inlineStr">
-        <is>
-          <t>Mua PC máy tính+ chuột (Mouse)</t>
-        </is>
-      </c>
+      <c r="S117" s="200" t="n"/>
       <c r="T117" s="201" t="n"/>
       <c r="U117" s="245" t="n"/>
       <c r="V117" s="245" t="n"/>
@@ -20777,9 +20449,7 @@
     </row>
     <row r="118" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A118" s="225" t="n"/>
-      <c r="B118" s="179" t="n">
-        <v>5005026371</v>
-      </c>
+      <c r="B118" s="179" t="n"/>
       <c r="C118" s="182">
         <f>IFERROR(IF(VLOOKUP($B118,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B118,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -20805,11 +20475,7 @@
         <f>SUM(F118:Q118)</f>
         <v/>
       </c>
-      <c r="S118" s="200" t="inlineStr">
-        <is>
-          <t>Libra2機</t>
-        </is>
-      </c>
+      <c r="S118" s="200" t="n"/>
       <c r="T118" s="201" t="n"/>
       <c r="U118" s="245" t="n"/>
       <c r="V118" s="245" t="n"/>
@@ -20817,9 +20483,7 @@
     </row>
     <row r="119" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A119" s="225" t="n"/>
-      <c r="B119" s="179" t="n">
-        <v>5005026371</v>
-      </c>
+      <c r="B119" s="179" t="n"/>
       <c r="C119" s="182">
         <f>IFERROR(IF(VLOOKUP($B119,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B119,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -20845,11 +20509,7 @@
         <f>SUM(F119:Q119)</f>
         <v/>
       </c>
-      <c r="S119" s="200" t="inlineStr">
-        <is>
-          <t>Pictor Color機</t>
-        </is>
-      </c>
+      <c r="S119" s="200" t="n"/>
       <c r="T119" s="201" t="n"/>
       <c r="U119" s="245" t="n"/>
       <c r="V119" s="245" t="n"/>
@@ -20857,9 +20517,7 @@
     </row>
     <row r="120" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A120" s="225" t="n"/>
-      <c r="B120" s="179" t="n">
-        <v>5005026371</v>
-      </c>
+      <c r="B120" s="179" t="n"/>
       <c r="C120" s="182">
         <f>IFERROR(IF(VLOOKUP($B120,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B120,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -20885,11 +20543,7 @@
         <f>SUM(F120:Q120)</f>
         <v/>
       </c>
-      <c r="S120" s="200" t="inlineStr">
-        <is>
-          <t>Polaris Next　MFP機</t>
-        </is>
-      </c>
+      <c r="S120" s="200" t="n"/>
       <c r="T120" s="201" t="n"/>
       <c r="U120" s="245" t="n"/>
       <c r="V120" s="245" t="n"/>
@@ -20897,9 +20551,7 @@
     </row>
     <row r="121" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A121" s="225" t="n"/>
-      <c r="B121" s="179" t="n">
-        <v>5005026371</v>
-      </c>
+      <c r="B121" s="179" t="n"/>
       <c r="C121" s="182">
         <f>IFERROR(IF(VLOOKUP($B121,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B121,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -20925,11 +20577,7 @@
         <f>SUM(F121:Q121)</f>
         <v/>
       </c>
-      <c r="S121" s="200" t="inlineStr">
-        <is>
-          <t>マウス</t>
-        </is>
-      </c>
+      <c r="S121" s="200" t="n"/>
       <c r="T121" s="201" t="n"/>
       <c r="U121" s="245" t="n"/>
       <c r="V121" s="245" t="n"/>
@@ -20965,9 +20613,7 @@
     </row>
     <row r="123" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A123" s="225" t="n"/>
-      <c r="B123" s="179" t="n">
-        <v>5005046282</v>
-      </c>
+      <c r="B123" s="179" t="n"/>
       <c r="C123" s="182">
         <f>IFERROR(IF(VLOOKUP($B123,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B123,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -20993,11 +20639,7 @@
         <f>SUM(F123:Q123)</f>
         <v/>
       </c>
-      <c r="S123" s="200" t="inlineStr">
-        <is>
-          <t>マウス</t>
-        </is>
-      </c>
+      <c r="S123" s="200" t="n"/>
       <c r="T123" s="201" t="n"/>
       <c r="U123" s="245" t="n"/>
       <c r="V123" s="245" t="n"/>
@@ -21005,9 +20647,7 @@
     </row>
     <row r="124" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A124" s="225" t="n"/>
-      <c r="B124" s="179" t="n">
-        <v>5005046282</v>
-      </c>
+      <c r="B124" s="179" t="n"/>
       <c r="C124" s="182">
         <f>IFERROR(IF(VLOOKUP($B124,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B124,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -21041,9 +20681,7 @@
     </row>
     <row r="125" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A125" s="225" t="n"/>
-      <c r="B125" s="179" t="n">
-        <v>5005046282</v>
-      </c>
+      <c r="B125" s="179" t="n"/>
       <c r="C125" s="182">
         <f>IFERROR(IF(VLOOKUP($B125,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B125,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -21105,9 +20743,7 @@
     </row>
     <row r="127" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A127" s="225" t="n"/>
-      <c r="B127" s="179" t="n">
-        <v>5005076281</v>
-      </c>
+      <c r="B127" s="179" t="n"/>
       <c r="C127" s="182">
         <f>IFERROR(IF(VLOOKUP($B127,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B127,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -21133,11 +20769,7 @@
         <f>SUM(F127:Q127)</f>
         <v/>
       </c>
-      <c r="S127" s="200" t="inlineStr">
-        <is>
-          <t>DECLARATION FEE (P)/通関費</t>
-        </is>
-      </c>
+      <c r="S127" s="200" t="n"/>
       <c r="T127" s="201" t="n"/>
       <c r="U127" s="245" t="n"/>
       <c r="V127" s="245" t="n"/>
@@ -21145,9 +20777,7 @@
     </row>
     <row r="128" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A128" s="225" t="n"/>
-      <c r="B128" s="179" t="n">
-        <v>5005076283</v>
-      </c>
+      <c r="B128" s="179" t="n"/>
       <c r="C128" s="182">
         <f>IFERROR(IF(VLOOKUP($B128,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B128,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -21173,11 +20803,7 @@
         <f>SUM(F128:Q128)</f>
         <v/>
       </c>
-      <c r="S128" s="200" t="inlineStr">
-        <is>
-          <t>輸送費DPデータ</t>
-        </is>
-      </c>
+      <c r="S128" s="200" t="n"/>
       <c r="T128" s="201" t="n"/>
       <c r="U128" s="245" t="n"/>
       <c r="V128" s="245" t="n"/>
@@ -21185,9 +20811,7 @@
     </row>
     <row r="129" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A129" s="225" t="n"/>
-      <c r="B129" s="179" t="n">
-        <v>5005076281</v>
-      </c>
+      <c r="B129" s="179" t="n"/>
       <c r="C129" s="182">
         <f>IFERROR(IF(VLOOKUP($B129,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B129,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -21213,11 +20837,7 @@
         <f>SUM(F129:Q129)</f>
         <v/>
       </c>
-      <c r="S129" s="200" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DECLARATION FEE (P)/通関費 </t>
-        </is>
-      </c>
+      <c r="S129" s="200" t="n"/>
       <c r="T129" s="201" t="n"/>
       <c r="U129" s="245" t="n"/>
       <c r="V129" s="245" t="n"/>
@@ -21225,9 +20845,7 @@
     </row>
     <row r="130" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A130" s="225" t="n"/>
-      <c r="B130" s="179" t="n">
-        <v>5005076289</v>
-      </c>
+      <c r="B130" s="179" t="n"/>
       <c r="C130" s="182">
         <f>IFERROR(IF(VLOOKUP($B130,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B130,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -21253,11 +20871,7 @@
         <f>SUM(F130:Q130)</f>
         <v/>
       </c>
-      <c r="S130" s="200" t="inlineStr">
-        <is>
-          <t>COURIER CHARGES (P)</t>
-        </is>
-      </c>
+      <c r="S130" s="200" t="n"/>
       <c r="T130" s="201" t="n"/>
       <c r="U130" s="245" t="n"/>
       <c r="V130" s="245" t="n"/>
@@ -21265,9 +20879,7 @@
     </row>
     <row r="131" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A131" s="225" t="n"/>
-      <c r="B131" s="179" t="n">
-        <v>5005076284</v>
-      </c>
+      <c r="B131" s="179" t="n"/>
       <c r="C131" s="182">
         <f>IFERROR(IF(VLOOKUP($B131,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B131,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -21293,11 +20905,7 @@
         <f>SUM(F131:Q131)</f>
         <v/>
       </c>
-      <c r="S131" s="200" t="inlineStr">
-        <is>
-          <t>IMPORT BOAT FEE (P)</t>
-        </is>
-      </c>
+      <c r="S131" s="200" t="n"/>
       <c r="T131" s="201" t="n"/>
       <c r="U131" s="245" t="n"/>
       <c r="V131" s="245" t="n"/>
@@ -21339,9 +20947,7 @@
     </row>
     <row r="133" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A133" s="225" t="n"/>
-      <c r="B133" s="179" t="n">
-        <v>5004086293</v>
-      </c>
+      <c r="B133" s="179" t="n"/>
       <c r="C133" s="182">
         <f>IFERROR(IF(VLOOKUP($B133,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B133,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -21367,11 +20973,7 @@
         <f>SUM(F133:Q133)</f>
         <v/>
       </c>
-      <c r="S133" s="200" t="inlineStr">
-        <is>
-          <t>JLPT試験費用、TOEIC受験費用/Phí đi thi JLPT, TOEIC</t>
-        </is>
-      </c>
+      <c r="S133" s="200" t="n"/>
       <c r="T133" s="201" t="n"/>
       <c r="U133" s="245" t="n"/>
       <c r="V133" s="245" t="n"/>
@@ -21379,9 +20981,7 @@
     </row>
     <row r="134" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A134" s="225" t="n"/>
-      <c r="B134" s="179" t="n">
-        <v>5004086293</v>
-      </c>
+      <c r="B134" s="179" t="n"/>
       <c r="C134" s="182">
         <f>IFERROR(IF(VLOOKUP($B134,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B134,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -21415,9 +21015,7 @@
     </row>
     <row r="135" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A135" s="225" t="n"/>
-      <c r="B135" s="179" t="n">
-        <v>5004086293</v>
-      </c>
+      <c r="B135" s="179" t="n"/>
       <c r="C135" s="182">
         <f>IFERROR(IF(VLOOKUP($B135,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B135,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -21485,9 +21083,7 @@
     </row>
     <row r="137" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A137" s="225" t="n"/>
-      <c r="B137" s="179" t="n">
-        <v>5005246286</v>
-      </c>
+      <c r="B137" s="179" t="n"/>
       <c r="C137" s="182">
         <f>IFERROR(IF(VLOOKUP($B137,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B137,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -21513,11 +21109,7 @@
         <f>SUM(F137:Q137)</f>
         <v/>
       </c>
-      <c r="S137" s="200" t="inlineStr">
-        <is>
-          <t>出向者の書類申請費/Chi phí làm giấy tờ cho người biệt phái</t>
-        </is>
-      </c>
+      <c r="S137" s="200" t="n"/>
       <c r="T137" s="201" t="n"/>
       <c r="U137" s="245" t="n"/>
       <c r="V137" s="245" t="n"/>
@@ -21525,9 +21117,7 @@
     </row>
     <row r="138" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A138" s="225" t="n"/>
-      <c r="B138" s="179" t="n">
-        <v>5005246286</v>
-      </c>
+      <c r="B138" s="179" t="n"/>
       <c r="C138" s="182">
         <f>IFERROR(IF(VLOOKUP($B138,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B138,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -21561,9 +21151,7 @@
     </row>
     <row r="139" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A139" s="225" t="n"/>
-      <c r="B139" s="179" t="n">
-        <v>5005246286</v>
-      </c>
+      <c r="B139" s="179" t="n"/>
       <c r="C139" s="182">
         <f>IFERROR(IF(VLOOKUP($B139,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B139,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -21597,9 +21185,7 @@
     </row>
     <row r="140" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A140" s="225" t="n"/>
-      <c r="B140" s="179" t="n">
-        <v>5005246286</v>
-      </c>
+      <c r="B140" s="179" t="n"/>
       <c r="C140" s="182">
         <f>IFERROR(IF(VLOOKUP($B140,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B140,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -21633,9 +21219,7 @@
     </row>
     <row r="141" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A141" s="225" t="n"/>
-      <c r="B141" s="179" t="n">
-        <v>5005246286</v>
-      </c>
+      <c r="B141" s="179" t="n"/>
       <c r="C141" s="182">
         <f>IFERROR(IF(VLOOKUP($B141,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B141,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -21669,9 +21253,7 @@
     </row>
     <row r="142" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A142" s="225" t="n"/>
-      <c r="B142" s="179" t="n">
-        <v>5005246286</v>
-      </c>
+      <c r="B142" s="179" t="n"/>
       <c r="C142" s="182">
         <f>IFERROR(IF(VLOOKUP($B142,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B142,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -21705,9 +21287,7 @@
     </row>
     <row r="143" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A143" s="225" t="n"/>
-      <c r="B143" s="179" t="n">
-        <v>5005246286</v>
-      </c>
+      <c r="B143" s="179" t="n"/>
       <c r="C143" s="182">
         <f>IFERROR(IF(VLOOKUP($B143,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B143,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -21741,9 +21321,7 @@
     </row>
     <row r="144" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A144" s="225" t="n"/>
-      <c r="B144" s="179" t="n">
-        <v>5005246286</v>
-      </c>
+      <c r="B144" s="179" t="n"/>
       <c r="C144" s="182">
         <f>IFERROR(IF(VLOOKUP($B144,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B144,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -21777,9 +21355,7 @@
     </row>
     <row r="145" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A145" s="225" t="n"/>
-      <c r="B145" s="179" t="n">
-        <v>5005246286</v>
-      </c>
+      <c r="B145" s="179" t="n"/>
       <c r="C145" s="182">
         <f>IFERROR(IF(VLOOKUP($B145,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B145,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -21813,9 +21389,7 @@
     </row>
     <row r="146" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A146" s="225" t="n"/>
-      <c r="B146" s="179" t="n">
-        <v>5005246286</v>
-      </c>
+      <c r="B146" s="179" t="n"/>
       <c r="C146" s="182">
         <f>IFERROR(IF(VLOOKUP($B146,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B146,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -21849,9 +21423,7 @@
     </row>
     <row r="147" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A147" s="225" t="n"/>
-      <c r="B147" s="179" t="n">
-        <v>5005246286</v>
-      </c>
+      <c r="B147" s="179" t="n"/>
       <c r="C147" s="182">
         <f>IFERROR(IF(VLOOKUP($B147,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B147,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -21919,9 +21491,7 @@
     </row>
     <row r="149" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A149" s="225" t="n"/>
-      <c r="B149" s="179" t="n">
-        <v>5005116291</v>
-      </c>
+      <c r="B149" s="179" t="n"/>
       <c r="C149" s="182">
         <f>IFERROR(IF(VLOOKUP($B149,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B149,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -21947,11 +21517,7 @@
         <f>SUM(F149:Q149)</f>
         <v/>
       </c>
-      <c r="S149" s="200" t="inlineStr">
-        <is>
-          <t>日本語受験の交通費/Chi phí đi lại đi thi tiếng nhật</t>
-        </is>
-      </c>
+      <c r="S149" s="200" t="n"/>
       <c r="T149" s="201" t="n"/>
       <c r="U149" s="245" t="n"/>
       <c r="V149" s="245" t="n"/>
@@ -21959,9 +21525,7 @@
     </row>
     <row r="150" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A150" s="225" t="n"/>
-      <c r="B150" s="179" t="n">
-        <v>5005116291</v>
-      </c>
+      <c r="B150" s="179" t="n"/>
       <c r="C150" s="182">
         <f>IFERROR(IF(VLOOKUP($B150,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B150,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -21987,11 +21551,7 @@
         <f>SUM(F150:Q150)</f>
         <v/>
       </c>
-      <c r="S150" s="200" t="inlineStr">
-        <is>
-          <t>VN内出張食事代/Tiền ăn khi đi công tác trong nước</t>
-        </is>
-      </c>
+      <c r="S150" s="200" t="n"/>
       <c r="T150" s="201" t="n"/>
       <c r="U150" s="245" t="n"/>
       <c r="V150" s="245" t="n"/>
@@ -21999,9 +21559,7 @@
     </row>
     <row r="151" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A151" s="225" t="n"/>
-      <c r="B151" s="179" t="n">
-        <v>5005116291</v>
-      </c>
+      <c r="B151" s="179" t="n"/>
       <c r="C151" s="182">
         <f>IFERROR(IF(VLOOKUP($B151,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B151,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -22027,11 +21585,7 @@
         <f>SUM(F151:Q151)</f>
         <v/>
       </c>
-      <c r="S151" s="200" t="inlineStr">
-        <is>
-          <t>VN内出張日当/Công tác phí khi đi công tác trong nước</t>
-        </is>
-      </c>
+      <c r="S151" s="200" t="n"/>
       <c r="T151" s="201" t="n"/>
       <c r="U151" s="245" t="n"/>
       <c r="V151" s="245" t="n"/>
@@ -22039,9 +21593,7 @@
     </row>
     <row r="152" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A152" s="225" t="n"/>
-      <c r="B152" s="179" t="n">
-        <v>5005116291</v>
-      </c>
+      <c r="B152" s="179" t="n"/>
       <c r="C152" s="182">
         <f>IFERROR(IF(VLOOKUP($B152,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B152,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -22067,11 +21619,7 @@
         <f>SUM(F152:Q152)</f>
         <v/>
       </c>
-      <c r="S152" s="200" t="inlineStr">
-        <is>
-          <t>VN内出張交通費/Tiền đi lại khi đi công tác trong nước</t>
-        </is>
-      </c>
+      <c r="S152" s="200" t="n"/>
       <c r="T152" s="201" t="n"/>
       <c r="U152" s="245" t="n"/>
       <c r="V152" s="245" t="n"/>
@@ -22141,9 +21689,7 @@
     </row>
     <row r="155" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A155" s="225" t="n"/>
-      <c r="B155" s="179" t="n">
-        <v>5005116292</v>
-      </c>
+      <c r="B155" s="179" t="n"/>
       <c r="C155" s="182">
         <f>IFERROR(IF(VLOOKUP($B155,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B155,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -22169,11 +21715,7 @@
         <f>SUM(F155:Q155)</f>
         <v/>
       </c>
-      <c r="S155" s="200" t="inlineStr">
-        <is>
-          <t>往復航空運賃/Tiền vé máy bay</t>
-        </is>
-      </c>
+      <c r="S155" s="200" t="n"/>
       <c r="T155" s="201" t="n"/>
       <c r="U155" s="245" t="n"/>
       <c r="V155" s="245" t="n"/>
@@ -22181,9 +21723,7 @@
     </row>
     <row r="156" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A156" s="225" t="n"/>
-      <c r="B156" s="179" t="n">
-        <v>5005116292</v>
-      </c>
+      <c r="B156" s="179" t="n"/>
       <c r="C156" s="182">
         <f>IFERROR(IF(VLOOKUP($B156,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B156,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -22209,11 +21749,7 @@
         <f>SUM(F156:Q156)</f>
         <v/>
       </c>
-      <c r="S156" s="200" t="inlineStr">
-        <is>
-          <t>日本で国際日当/Tiền công tác phí đi công tác JP</t>
-        </is>
-      </c>
+      <c r="S156" s="200" t="n"/>
       <c r="T156" s="201" t="n"/>
       <c r="U156" s="245" t="n"/>
       <c r="V156" s="245" t="n"/>
@@ -22221,9 +21757,7 @@
     </row>
     <row r="157" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A157" s="225" t="n"/>
-      <c r="B157" s="179" t="n">
-        <v>5005116292</v>
-      </c>
+      <c r="B157" s="179" t="n"/>
       <c r="C157" s="182">
         <f>IFERROR(IF(VLOOKUP($B157,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B157,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -22249,11 +21783,7 @@
         <f>SUM(F157:Q157)</f>
         <v/>
       </c>
-      <c r="S157" s="200" t="inlineStr">
-        <is>
-          <t>日本で現地交通費、通信費/Phí đi lại, liên lạc tại JP</t>
-        </is>
-      </c>
+      <c r="S157" s="200" t="n"/>
       <c r="T157" s="201" t="n"/>
       <c r="U157" s="245" t="n"/>
       <c r="V157" s="245" t="n"/>
@@ -22261,9 +21791,7 @@
     </row>
     <row r="158" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A158" s="225" t="n"/>
-      <c r="B158" s="179" t="n">
-        <v>5005116292</v>
-      </c>
+      <c r="B158" s="179" t="n"/>
       <c r="C158" s="182">
         <f>IFERROR(IF(VLOOKUP($B158,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B158,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -22289,11 +21817,7 @@
         <f>SUM(F158:Q158)</f>
         <v/>
       </c>
-      <c r="S158" s="200" t="inlineStr">
-        <is>
-          <t>写真撮影料金＋公証費用、大使館の手数料、VISA取得費用、保険料/Tiền chụp ảnh+công chứng, đại sứ quán, làm VISA, bảo hiểm</t>
-        </is>
-      </c>
+      <c r="S158" s="200" t="n"/>
       <c r="T158" s="201" t="n"/>
       <c r="U158" s="245" t="n"/>
       <c r="V158" s="245" t="n"/>
@@ -22301,9 +21825,7 @@
     </row>
     <row r="159" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A159" s="225" t="n"/>
-      <c r="B159" s="179" t="n">
-        <v>5005116292</v>
-      </c>
+      <c r="B159" s="179" t="n"/>
       <c r="C159" s="182">
         <f>IFERROR(IF(VLOOKUP($B159,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B159,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -22329,11 +21851,7 @@
         <f>SUM(F159:Q159)</f>
         <v/>
       </c>
-      <c r="S159" s="200" t="inlineStr">
-        <is>
-          <t>宿泊費/Tiền khách sạn</t>
-        </is>
-      </c>
+      <c r="S159" s="200" t="n"/>
       <c r="T159" s="201" t="n"/>
       <c r="U159" s="245" t="n"/>
       <c r="V159" s="245" t="n"/>
@@ -22341,9 +21859,7 @@
     </row>
     <row r="160" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A160" s="225" t="n"/>
-      <c r="B160" s="179" t="n">
-        <v>5005116292</v>
-      </c>
+      <c r="B160" s="179" t="n"/>
       <c r="C160" s="182">
         <f>IFERROR(IF(VLOOKUP($B160,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B160,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -22377,9 +21893,7 @@
     </row>
     <row r="161" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A161" s="225" t="n"/>
-      <c r="B161" s="179" t="n">
-        <v>5005116292</v>
-      </c>
+      <c r="B161" s="179" t="n"/>
       <c r="C161" s="182">
         <f>IFERROR(IF(VLOOKUP($B161,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B161,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -22413,9 +21927,7 @@
     </row>
     <row r="162" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A162" s="225" t="n"/>
-      <c r="B162" s="179" t="n">
-        <v>5005116292</v>
-      </c>
+      <c r="B162" s="179" t="n"/>
       <c r="C162" s="182">
         <f>IFERROR(IF(VLOOKUP($B162,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B162,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -22449,9 +21961,7 @@
     </row>
     <row r="163" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A163" s="225" t="n"/>
-      <c r="B163" s="179" t="n">
-        <v>5005116292</v>
-      </c>
+      <c r="B163" s="179" t="n"/>
       <c r="C163" s="182">
         <f>IFERROR(IF(VLOOKUP($B163,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B163,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -22485,9 +21995,7 @@
     </row>
     <row r="164" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A164" s="225" t="n"/>
-      <c r="B164" s="179" t="n">
-        <v>5005116292</v>
-      </c>
+      <c r="B164" s="179" t="n"/>
       <c r="C164" s="182">
         <f>IFERROR(IF(VLOOKUP($B164,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B164,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -22555,9 +22063,7 @@
     </row>
     <row r="166" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A166" s="225" t="n"/>
-      <c r="B166" s="179" t="n">
-        <v>9114120009</v>
-      </c>
+      <c r="B166" s="179" t="n"/>
       <c r="C166" s="182">
         <f>IFERROR(IF(VLOOKUP($B166,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B166,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -22583,11 +22089,7 @@
         <f>SUM(F166:Q166)</f>
         <v/>
       </c>
-      <c r="S166" s="200" t="inlineStr">
-        <is>
-          <t>在庫金利/Lãi tồn kho</t>
-        </is>
-      </c>
+      <c r="S166" s="200" t="n"/>
       <c r="T166" s="201" t="n"/>
       <c r="U166" s="245" t="n"/>
       <c r="V166" s="245" t="n"/>

</xml_diff>

<commit_message>
fix: harden fiscal export reconciliation
</commit_message>
<xml_diff>
--- a/docs/MP2027/FORM.xlsx
+++ b/docs/MP2027/FORM.xlsx
@@ -8365,6 +8365,7 @@
         <v/>
       </c>
     </row>
+    <row r="90"/>
     <row r="91">
       <c r="B91" s="16" t="inlineStr">
         <is>
@@ -15935,9 +15936,7 @@
       <c r="T4" s="96" t="n"/>
     </row>
     <row r="5" ht="13.5" customHeight="1" thickBot="1">
-      <c r="B5" s="160" t="n">
-        <v>1412000006</v>
-      </c>
+      <c r="B5" s="160" t="n"/>
       <c r="C5" s="7">
         <f>VLOOKUP($B$5,原価センタ!$A:$E,2,0)</f>
         <v/>
@@ -17751,9 +17750,7 @@
     </row>
     <row r="46" ht="12.95" customFormat="1" customHeight="1" s="177">
       <c r="A46" s="211" t="n"/>
-      <c r="B46" s="166" t="n">
-        <v>5005056281</v>
-      </c>
+      <c r="B46" s="166" t="n"/>
       <c r="C46" s="169">
         <f>IFERROR(IF(VLOOKUP($B46,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B46,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -17779,16 +17776,8 @@
         <f>SUM(F46:Q46)</f>
         <v/>
       </c>
-      <c r="S46" s="187" t="inlineStr">
-        <is>
-          <t>ガス代/Tiền gas</t>
-        </is>
-      </c>
-      <c r="T46" s="188" t="inlineStr">
-        <is>
-          <t>business_key=recurring_admin_gas</t>
-        </is>
-      </c>
+      <c r="S46" s="187" t="n"/>
+      <c r="T46" s="188" t="n"/>
       <c r="U46" s="231" t="n"/>
       <c r="V46" s="231" t="n"/>
       <c r="W46" s="231" t="n"/>
@@ -17829,9 +17818,7 @@
     </row>
     <row r="48" ht="12.95" customFormat="1" customHeight="1" s="177">
       <c r="A48" s="211" t="n"/>
-      <c r="B48" s="166" t="n">
-        <v>5005016372</v>
-      </c>
+      <c r="B48" s="166" t="n"/>
       <c r="C48" s="169">
         <f>IFERROR(IF(VLOOKUP($B48,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B48,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -17857,25 +17844,15 @@
         <f>SUM(F48:Q48)</f>
         <v/>
       </c>
-      <c r="S48" s="187" t="inlineStr">
-        <is>
-          <t>Hand wash/Nước rửa tay</t>
-        </is>
-      </c>
-      <c r="T48" s="188" t="inlineStr">
-        <is>
-          <t>business_key=recurring_admin_handwash</t>
-        </is>
-      </c>
+      <c r="S48" s="187" t="n"/>
+      <c r="T48" s="188" t="n"/>
       <c r="U48" s="231" t="n"/>
       <c r="V48" s="231" t="n"/>
       <c r="W48" s="231" t="n"/>
     </row>
     <row r="49" ht="12.95" customFormat="1" customHeight="1" s="177">
       <c r="A49" s="211" t="n"/>
-      <c r="B49" s="166" t="n">
-        <v>5005016372</v>
-      </c>
+      <c r="B49" s="166" t="n"/>
       <c r="C49" s="169">
         <f>IFERROR(IF(VLOOKUP($B49,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B49,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -17901,16 +17878,8 @@
         <f>SUM(F49:Q49)</f>
         <v/>
       </c>
-      <c r="S49" s="187" t="inlineStr">
-        <is>
-          <t>Toilet paper/Giấy vệ sinh</t>
-        </is>
-      </c>
-      <c r="T49" s="188" t="inlineStr">
-        <is>
-          <t>business_key=recurring_admin_toilet_paper</t>
-        </is>
-      </c>
+      <c r="S49" s="187" t="n"/>
+      <c r="T49" s="188" t="n"/>
       <c r="U49" s="231" t="n"/>
       <c r="V49" s="231" t="n"/>
       <c r="W49" s="231" t="n"/>
@@ -17942,9 +17911,7 @@
     </row>
     <row r="51" ht="12.95" customFormat="1" customHeight="1" s="177">
       <c r="A51" s="211" t="n"/>
-      <c r="B51" s="166" t="n">
-        <v>5005246286</v>
-      </c>
+      <c r="B51" s="166" t="n"/>
       <c r="C51" s="169">
         <f>IFERROR(IF(VLOOKUP($B51,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B51,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -17970,16 +17937,8 @@
         <f>SUM(F51:Q51)</f>
         <v/>
       </c>
-      <c r="S51" s="187" t="inlineStr">
-        <is>
-          <t>cleaning fee/Chi phí làm sạch</t>
-        </is>
-      </c>
-      <c r="T51" s="188" t="inlineStr">
-        <is>
-          <t>business_key=recurring_admin_cleaning</t>
-        </is>
-      </c>
+      <c r="S51" s="187" t="n"/>
+      <c r="T51" s="188" t="n"/>
       <c r="U51" s="231" t="n"/>
       <c r="V51" s="231" t="n"/>
       <c r="W51" s="231" t="n"/>
@@ -50121,7 +50080,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:S55"/>
+  <dimension ref="A1:S55"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="3.125" customWidth="1" style="47" min="1" max="1"/>
@@ -60778,12 +60737,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:B14"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="9" customWidth="1" style="233" min="2" max="2"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="A2" s="113" t="inlineStr">
         <is>

</xml_diff>